<commit_message>
feat: implement dataset curation utilities and update validation reporting with corrected candidate metadata (lol ai) BUT I DID EDA
</commit_message>
<xml_diff>
--- a/data/stories_cleaned.xlsx
+++ b/data/stories_cleaned.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:T69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,7 +479,42 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Unnamed: 12</t>
+          <t>mal_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>mal_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>mal_popularity</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>mal_members</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>mal_favorites</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>mal_genres</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>mal_themes</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>serialization</t>
         </is>
       </c>
     </row>
@@ -538,7 +573,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>31499</v>
+      </c>
+      <c r="N2" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="O2" t="n">
+        <v>45</v>
+      </c>
+      <c r="P2" t="n">
+        <v>210467</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>13517</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Shounen Jump (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -595,7 +659,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>103851</v>
+      </c>
+      <c r="N3" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="O3" t="n">
+        <v>68</v>
+      </c>
+      <c r="P3" t="n">
+        <v>179115</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>10698</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Award Winning; Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -652,7 +745,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>51309</v>
+      </c>
+      <c r="N4" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2990</v>
+      </c>
+      <c r="P4" t="n">
+        <v>8645</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>74</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Dragon Age</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -709,7 +831,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>7519</v>
+      </c>
+      <c r="N5" t="n">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="O5" t="n">
+        <v>140</v>
+      </c>
+      <c r="P5" t="n">
+        <v>115444</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>9280</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Comedy; Fantasy; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Harem; Otaku Culture; School</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Shounen Sunday</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -745,7 +896,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Shounen</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -767,7 +918,34 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>269</v>
+        <v>137</v>
+      </c>
+      <c r="N6" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="O6" t="n">
+        <v>4445</v>
+      </c>
+      <c r="P6" t="n">
+        <v>5815</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>79</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Mystery</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Adult Cast; Super Power</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Ultra Jump</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -825,7 +1003,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="O7" t="n">
+        <v>22441</v>
+      </c>
+      <c r="P7" t="n">
+        <v>726</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Comedy; Ecchi</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Dengeki Comic Gao!</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -882,7 +1085,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>894</v>
+      </c>
+      <c r="N8" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="O8" t="n">
+        <v>164</v>
+      </c>
+      <c r="P8" t="n">
+        <v>102239</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3621</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Fantasy; Romance; Supernatural; Ecchi</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Harem; School; Vampire</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Shounen Jump (Monthly)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -939,7 +1171,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>40171</v>
+      </c>
+      <c r="N9" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="O9" t="n">
+        <v>232</v>
+      </c>
+      <c r="P9" t="n">
+        <v>77179</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>4198</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Love Polygon; School</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -996,7 +1257,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>7149</v>
+      </c>
+      <c r="N10" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="O10" t="n">
+        <v>729</v>
+      </c>
+      <c r="P10" t="n">
+        <v>29497</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>822</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Love Polygon; School</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1032,7 +1322,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Seinen</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1053,7 +1343,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>36873</v>
+      </c>
+      <c r="N11" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1831</v>
+      </c>
+      <c r="P11" t="n">
+        <v>13705</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>204</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Dengeki Daioh</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1110,7 +1425,36 @@
           <t>Visual Novel</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>18245</v>
+      </c>
+      <c r="N12" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1060</v>
+      </c>
+      <c r="P12" t="n">
+        <v>268475</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>3523</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Love Polygon; Music</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Leaf</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1167,7 +1511,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>8483</v>
+      </c>
+      <c r="N13" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="O13" t="n">
+        <v>247</v>
+      </c>
+      <c r="P13" t="n">
+        <v>73485</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>4224</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Drama; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Love Polygon; School</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1224,7 +1597,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>430</v>
+      </c>
+      <c r="N14" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="O14" t="n">
+        <v>380</v>
+      </c>
+      <c r="P14" t="n">
+        <v>51767</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1849</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Romance; Sports; Ecchi</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1281,7 +1679,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>70941</v>
+      </c>
+      <c r="N15" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="O15" t="n">
+        <v>116</v>
+      </c>
+      <c r="P15" t="n">
+        <v>129686</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>7123</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Love Polygon; School</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1338,7 +1765,28 @@
           <t>Anime Original</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>3196</v>
+      </c>
+      <c r="N16" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="O16" t="n">
+        <v>10585</v>
+      </c>
+      <c r="P16" t="n">
+        <v>3727</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>11</v>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Nippon Animation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1395,7 +1843,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>482</v>
+      </c>
+      <c r="N17" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="O17" t="n">
+        <v>8521</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2764</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>11</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Princess</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1452,7 +1925,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>91514</v>
+      </c>
+      <c r="N18" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="O18" t="n">
+        <v>270</v>
+      </c>
+      <c r="P18" t="n">
+        <v>69592</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3079</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1488,7 +1986,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Seinen</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1509,7 +2007,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>46716</v>
+      </c>
+      <c r="N19" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="O19" t="n">
+        <v>159</v>
+      </c>
+      <c r="P19" t="n">
+        <v>104485</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1917</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Comic REX</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1566,7 +2093,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>35003</v>
+      </c>
+      <c r="N20" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="O20" t="n">
+        <v>120</v>
+      </c>
+      <c r="P20" t="n">
+        <v>125373</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>5300</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Comedy; Mystery; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1623,7 +2179,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>23390</v>
+      </c>
+      <c r="N21" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="O21" t="n">
+        <v>4</v>
+      </c>
+      <c r="P21" t="n">
+        <v>696181</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>69929</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Action; Award Winning; Drama; Suspense</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Gore; Military; Survival</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Bessatsu Shounen Magazine</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1680,7 +2265,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>75</v>
+      </c>
+      <c r="N22" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1725</v>
+      </c>
+      <c r="P22" t="n">
+        <v>14348</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>323</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Young Animal</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1716,7 +2326,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Shounen</t>
+          <t>Shoujo</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1737,7 +2347,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>124</v>
+      </c>
+      <c r="N23" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="O23" t="n">
+        <v>1053</v>
+      </c>
+      <c r="P23" t="n">
+        <v>21330</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>351</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Sci-Fi; Slice of Life</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Stencil</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1794,7 +2429,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>696</v>
+      </c>
+      <c r="N24" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="O24" t="n">
+        <v>638</v>
+      </c>
+      <c r="P24" t="n">
+        <v>33276</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>1916</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Harem; Parody</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Shounen Sunday</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1830,7 +2494,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shoujo</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1851,7 +2515,28 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>1089</v>
+      </c>
+      <c r="N25" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="O25" t="n">
+        <v>12503</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1718</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>26</v>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1908,7 +2593,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>902</v>
+      </c>
+      <c r="N26" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="O26" t="n">
+        <v>6617</v>
+      </c>
+      <c r="P26" t="n">
+        <v>3744</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>38</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Boys Love; Drama; Slice of Life</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1965,7 +2675,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>18597</v>
+      </c>
+      <c r="N27" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="O27" t="n">
+        <v>207</v>
+      </c>
+      <c r="P27" t="n">
+        <v>87437</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>2441</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Comedy; Horror; Romance; Supernatural; Ecchi</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Bessatsu Shounen Magazine</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2001,7 +2736,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2022,7 +2757,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>22421</v>
+      </c>
+      <c r="N28" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="O28" t="n">
+        <v>22862</v>
+      </c>
+      <c r="P28" t="n">
+        <v>703</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>5</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Action; Adventure; Fantasy</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>CoroCoro Comic</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2058,7 +2818,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2079,7 +2839,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>37163</v>
+      </c>
+      <c r="N29" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="O29" t="n">
+        <v>3586</v>
+      </c>
+      <c r="P29" t="n">
+        <v>7202</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>146</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Fantasy; Romance; Sci-Fi</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>School; Urban Fantasy</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Shounen Ace</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2115,7 +2904,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2136,7 +2925,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>41021</v>
+      </c>
+      <c r="N30" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="O30" t="n">
+        <v>4119</v>
+      </c>
+      <c r="P30" t="n">
+        <v>6297</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>103</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Action; Fantasy; Ecchi</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>School; Urban Fantasy; Vampire</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2172,7 +2990,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2193,7 +3011,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>34553</v>
+      </c>
+      <c r="N31" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="O31" t="n">
+        <v>2913</v>
+      </c>
+      <c r="P31" t="n">
+        <v>8844</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>206</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Fantasy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2250,7 +3097,28 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>1733</v>
+      </c>
+      <c r="N32" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="O32" t="n">
+        <v>10257</v>
+      </c>
+      <c r="P32" t="n">
+        <v>2201</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>19</v>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Gangan Wing</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2286,7 +3154,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2307,7 +3175,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>56217</v>
+      </c>
+      <c r="N33" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="O33" t="n">
+        <v>5278</v>
+      </c>
+      <c r="P33" t="n">
+        <v>4828</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>58</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Action; Fantasy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2343,7 +3240,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2364,7 +3261,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>56249</v>
+      </c>
+      <c r="N34" t="n">
+        <v>7.26</v>
+      </c>
+      <c r="O34" t="n">
+        <v>7946</v>
+      </c>
+      <c r="P34" t="n">
+        <v>3021</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>31</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Action; Romance; Sci-Fi; Ecchi</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Harem; Mecha; School</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2400,7 +3326,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2421,7 +3347,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>51023</v>
+      </c>
+      <c r="N35" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="O35" t="n">
+        <v>2905</v>
+      </c>
+      <c r="P35" t="n">
+        <v>8869</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>66</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Action; Fantasy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Harem; School; Urban Fantasy</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Comic Alive</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2457,7 +3412,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2478,7 +3433,36 @@
           <t>Visual Novel</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>12175</v>
+      </c>
+      <c r="N36" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1064</v>
+      </c>
+      <c r="P36" t="n">
+        <v>267636</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>484</v>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>sprite</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2514,7 +3498,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2535,7 +3519,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>57201</v>
+      </c>
+      <c r="N37" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="O37" t="n">
+        <v>1223</v>
+      </c>
+      <c r="P37" t="n">
+        <v>19003</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>499</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Fantasy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>School; Urban Fantasy</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2571,7 +3584,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2592,7 +3605,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>3074</v>
+      </c>
+      <c r="N38" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="O38" t="n">
+        <v>2922</v>
+      </c>
+      <c r="P38" t="n">
+        <v>8821</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>209</v>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Action; Drama; Fantasy; Romance</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>School; Urban Fantasy</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2628,7 +3670,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2649,7 +3691,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>1154</v>
+      </c>
+      <c r="N39" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1996</v>
+      </c>
+      <c r="P39" t="n">
+        <v>12684</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>196</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Comedy; Fantasy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Harem; Isekai; School</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Comic Alive</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2685,7 +3756,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2706,7 +3777,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>92182</v>
+      </c>
+      <c r="N40" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="O40" t="n">
+        <v>752</v>
+      </c>
+      <c r="P40" t="n">
+        <v>28818</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>666</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Dengeki G's Comic</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2742,7 +3838,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2763,7 +3859,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>74697</v>
+      </c>
+      <c r="N41" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="O41" t="n">
+        <v>208</v>
+      </c>
+      <c r="P41" t="n">
+        <v>86970</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>6932</v>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Drama; Fantasy; Suspense</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Isekai; Psychological; Time Travel</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2799,7 +3924,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2820,7 +3945,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>14893</v>
+      </c>
+      <c r="N42" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="O42" t="n">
+        <v>283</v>
+      </c>
+      <c r="P42" t="n">
+        <v>67507</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>3305</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Mystery; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Mephisto</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2856,7 +4006,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2877,7 +4027,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="n">
+        <v>21621</v>
+      </c>
+      <c r="N43" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="O43" t="n">
+        <v>2025</v>
+      </c>
+      <c r="P43" t="n">
+        <v>12497</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>294</v>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2913,7 +4092,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2934,7 +4113,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>26613</v>
+      </c>
+      <c r="N44" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="O44" t="n">
+        <v>4642</v>
+      </c>
+      <c r="P44" t="n">
+        <v>5553</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>55</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2970,7 +4178,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2991,7 +4199,36 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>24822</v>
+      </c>
+      <c r="N45" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="O45" t="n">
+        <v>427</v>
+      </c>
+      <c r="P45" t="n">
+        <v>46683</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1025</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Action; Comedy; Fantasy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Harem; School</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Dragon Age</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3027,7 +4264,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3048,7 +4285,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>23881</v>
+      </c>
+      <c r="N46" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="O46" t="n">
+        <v>4666</v>
+      </c>
+      <c r="P46" t="n">
+        <v>5524</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>49</v>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Action; Romance; Sci-Fi</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3105,7 +4367,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="n">
+        <v>123602</v>
+      </c>
+      <c r="N47" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="O47" t="n">
+        <v>442</v>
+      </c>
+      <c r="P47" t="n">
+        <v>45656</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>546</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3162,7 +4449,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="n">
+        <v>133696</v>
+      </c>
+      <c r="N48" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="O48" t="n">
+        <v>946</v>
+      </c>
+      <c r="P48" t="n">
+        <v>23739</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>409</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Comedy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Adult Cast; Harem</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3219,7 +4535,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="n">
+        <v>134028</v>
+      </c>
+      <c r="N49" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="O49" t="n">
+        <v>869</v>
+      </c>
+      <c r="P49" t="n">
+        <v>25466</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>412</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Comedy; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3276,7 +4617,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="n">
+        <v>15578</v>
+      </c>
+      <c r="N50" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="O50" t="n">
+        <v>353</v>
+      </c>
+      <c r="P50" t="n">
+        <v>54241</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>1868</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Love Polygon; School</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Shounen Magazine (Weekly)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3333,7 +4703,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="n">
+        <v>26769</v>
+      </c>
+      <c r="N51" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="O51" t="n">
+        <v>422</v>
+      </c>
+      <c r="P51" t="n">
+        <v>46928</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>1510</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Romance; Slice of Life</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Young King OURs</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3369,7 +4764,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3390,7 +4785,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="n">
+        <v>28107</v>
+      </c>
+      <c r="N52" t="n">
+        <v>7.79</v>
+      </c>
+      <c r="O52" t="n">
+        <v>1823</v>
+      </c>
+      <c r="P52" t="n">
+        <v>13736</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>162</v>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Comedy; Romance; Slice of Life; Ecchi</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Dengeki G's Comic</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3426,7 +4846,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3447,7 +4867,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="n">
+        <v>25679</v>
+      </c>
+      <c r="N53" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="O53" t="n">
+        <v>1518</v>
+      </c>
+      <c r="P53" t="n">
+        <v>16057</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>119</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Comedy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Comic Alive</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3483,7 +4928,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3504,7 +4949,32 @@
           <t>Light Novel</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="n">
+        <v>3083</v>
+      </c>
+      <c r="N54" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="O54" t="n">
+        <v>508</v>
+      </c>
+      <c r="P54" t="n">
+        <v>40849</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>1845</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Sci-Fi; Supernatural</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>The Sneaker</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3561,7 +5031,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="n">
+        <v>17207</v>
+      </c>
+      <c r="N55" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="O55" t="n">
+        <v>553</v>
+      </c>
+      <c r="P55" t="n">
+        <v>37452</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>978</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Comedy; Mystery; Supernatural</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Gangan Joker</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3597,7 +5092,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3618,7 +5113,32 @@
           <t>Visual Novel</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
+      <c r="M56" t="n">
+        <v>2167</v>
+      </c>
+      <c r="N56" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="O56" t="n">
+        <v>95</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1520172</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>28868</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3654,7 +5174,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3675,7 +5195,32 @@
           <t>Visual Novel</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
+      <c r="M57" t="n">
+        <v>1530</v>
+      </c>
+      <c r="N57" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="O57" t="n">
+        <v>967</v>
+      </c>
+      <c r="P57" t="n">
+        <v>293280</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>4563</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Drama; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3711,7 +5256,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3732,7 +5277,32 @@
           <t>Visual Novel</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" t="n">
+        <v>101</v>
+      </c>
+      <c r="N58" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="O58" t="n">
+        <v>910</v>
+      </c>
+      <c r="P58" t="n">
+        <v>314420</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>2799</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Drama; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3789,7 +5359,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="n">
+        <v>1271</v>
+      </c>
+      <c r="N59" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="O59" t="n">
+        <v>458</v>
+      </c>
+      <c r="P59" t="n">
+        <v>44369</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>1109</v>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Hana to Yume</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3846,7 +5441,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="n">
+        <v>30</v>
+      </c>
+      <c r="N60" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O60" t="n">
+        <v>106</v>
+      </c>
+      <c r="P60" t="n">
+        <v>137419</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>8370</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Crossdressing; Reverse Harem; School</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>LaLa</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3903,7 +5527,36 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
+      <c r="M61" t="n">
+        <v>102</v>
+      </c>
+      <c r="N61" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="O61" t="n">
+        <v>91</v>
+      </c>
+      <c r="P61" t="n">
+        <v>152478</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>14919</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Award Winning; Drama; Romance; Supernatural</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Love Polygon; School</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Hana to Yume</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3960,7 +5613,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
+      <c r="M62" t="n">
+        <v>3378</v>
+      </c>
+      <c r="N62" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="O62" t="n">
+        <v>110</v>
+      </c>
+      <c r="P62" t="n">
+        <v>133024</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>5724</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Award Winning; Romance; Slice of Life</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Bessatsu Margaret</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4010,14 +5688,39 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>Manga</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr"/>
+      <c r="M63" t="n">
+        <v>31</v>
+      </c>
+      <c r="N63" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="O63" t="n">
+        <v>266</v>
+      </c>
+      <c r="P63" t="n">
+        <v>70369</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>2998</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Award Winning; Comedy; Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Bessatsu Margaret</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4074,7 +5777,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr"/>
+      <c r="M64" t="n">
+        <v>17</v>
+      </c>
+      <c r="N64" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="O64" t="n">
+        <v>488</v>
+      </c>
+      <c r="P64" t="n">
+        <v>42189</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>1648</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Comedy; Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>LaLa</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4110,7 +5838,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Shoujo</t>
+          <t>Seinen</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4131,7 +5859,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
+      <c r="M65" t="n">
+        <v>19007</v>
+      </c>
+      <c r="N65" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="O65" t="n">
+        <v>1131</v>
+      </c>
+      <c r="P65" t="n">
+        <v>20237</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>331</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Comedy; Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Young Jump</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4188,7 +5941,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
+      <c r="M66" t="n">
+        <v>1926</v>
+      </c>
+      <c r="N66" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="O66" t="n">
+        <v>405</v>
+      </c>
+      <c r="P66" t="n">
+        <v>49677</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>2247</v>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Romance; Ecchi</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4224,7 +6002,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Shoujo</t>
+          <t>Josei</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4245,7 +6023,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr"/>
+      <c r="M67" t="n">
+        <v>68675</v>
+      </c>
+      <c r="N67" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="O67" t="n">
+        <v>6615</v>
+      </c>
+      <c r="P67" t="n">
+        <v>3745</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>18</v>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Comedy; Romance</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Comic Gene</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4302,7 +6105,32 @@
           <t>Manga</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr"/>
+      <c r="M68" t="n">
+        <v>41847</v>
+      </c>
+      <c r="N68" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="O68" t="n">
+        <v>850</v>
+      </c>
+      <c r="P68" t="n">
+        <v>26073</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>535</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Adventure; Fantasy; Romance</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Hana to Yume</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4338,7 +6166,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Shounen</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4359,7 +6187,32 @@
           <t>Anime Original</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr"/>
+      <c r="M69" t="n">
+        <v>2926</v>
+      </c>
+      <c r="N69" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="O69" t="n">
+        <v>1455</v>
+      </c>
+      <c r="P69" t="n">
+        <v>193129</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>773</v>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Drama; Romance</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Doga Kobo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>